<commit_message>
Actualizacion de FastAPI con endpoints completos y corregidos
</commit_message>
<xml_diff>
--- a/Control_Inventario_Pole_Dance.xlsx
+++ b/Control_Inventario_Pole_Dance.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Winberthey Gaitan Hernandez\OneDrive - CENICANA\Escritorio\Academia\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cenicanaoff365-my.sharepoint.com/personal/iavar3_cenicanaoff365_onmicrosoft_com/Documents/Escritorio/Academia/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8F039D2-5B30-42AD-85ED-01D7E78216B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="17" documentId="13_ncr:1_{D8F039D2-5B30-42AD-85ED-01D7E78216B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DAD43FD3-F47E-4905-87FE-0927DD75E0EC}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="2" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28690" yWindow="-110" windowWidth="24220" windowHeight="13000" firstSheet="2" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="📊 Dashboard Control" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="300" uniqueCount="196">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="306" uniqueCount="199">
   <si>
     <t>PANEL DE CONTROL E INVENTARIOS - POLE DANCE ACADEMY</t>
   </si>
@@ -565,9 +565,6 @@
     <t>ACT-008</t>
   </si>
   <si>
-    <t>Sistema de Sonido Bluetooth 200W</t>
-  </si>
-  <si>
     <t>2025-01-12</t>
   </si>
   <si>
@@ -626,6 +623,18 @@
   </si>
   <si>
     <t>ACT-009</t>
+  </si>
+  <si>
+    <t>Barra / Pole Profesional Plateado</t>
+  </si>
+  <si>
+    <t>Espuma + casata</t>
+  </si>
+  <si>
+    <t>Colchoneta de Caída para Pole espuma + casata</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sistema de Sonido </t>
   </si>
 </sst>
 </file>
@@ -837,26 +846,30 @@
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="164" fontId="10" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="164" fontId="10" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="3" fontId="10" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -865,15 +878,11 @@
     <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -981,19 +990,19 @@
                 <c:formatCode>#,##0</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>1</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>1</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>2</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>1</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1189,13 +1198,13 @@
                 <c:formatCode>\$#,##0</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>175000</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>35000</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>85000</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>0</c:v>
@@ -1606,101 +1615,101 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="40" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="34" t="s">
+      <c r="A1" s="24" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="35"/>
-      <c r="C1" s="35"/>
-      <c r="D1" s="35"/>
-      <c r="E1" s="35"/>
-      <c r="F1" s="35"/>
-      <c r="G1" s="35"/>
-      <c r="H1" s="35"/>
-      <c r="I1" s="35"/>
+      <c r="B1" s="25"/>
+      <c r="C1" s="25"/>
+      <c r="D1" s="25"/>
+      <c r="E1" s="25"/>
+      <c r="F1" s="25"/>
+      <c r="G1" s="25"/>
+      <c r="H1" s="25"/>
+      <c r="I1" s="25"/>
     </row>
     <row r="3" spans="1:9" ht="26" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="33" t="s">
+      <c r="A3" s="32" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="24"/>
-      <c r="C3" s="24"/>
-      <c r="D3" s="24"/>
+      <c r="B3" s="27"/>
+      <c r="C3" s="27"/>
+      <c r="D3" s="27"/>
     </row>
     <row r="4" spans="1:9" ht="32" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="27" t="s">
+      <c r="A4" s="30" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="24"/>
-      <c r="C4" s="28" t="s">
+      <c r="B4" s="27"/>
+      <c r="C4" s="35" t="s">
         <v>3</v>
       </c>
-      <c r="D4" s="24"/>
+      <c r="D4" s="27"/>
     </row>
     <row r="5" spans="1:9" ht="22" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="27" t="s">
+      <c r="A5" s="30" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="24"/>
-      <c r="C5" s="23" t="str">
+      <c r="B5" s="27"/>
+      <c r="C5" s="31" t="str">
         <f>IFERROR(VLOOKUP(C4, '🏷️ Catálogo Productos'!A:C, 3, FALSE), "⚠️ Código no encontrado")</f>
         <v>Top Velvet Negro</v>
       </c>
-      <c r="D5" s="24"/>
+      <c r="D5" s="27"/>
     </row>
     <row r="6" spans="1:9" ht="22" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="27" t="s">
+      <c r="A6" s="30" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="24"/>
-      <c r="C6" s="23" t="str">
+      <c r="B6" s="27"/>
+      <c r="C6" s="31" t="str">
         <f>IFERROR(VLOOKUP(C4, '🏷️ Catálogo Productos'!A:D, 4, FALSE), "-")</f>
         <v>M</v>
       </c>
-      <c r="D6" s="24"/>
+      <c r="D6" s="27"/>
     </row>
     <row r="7" spans="1:9" ht="22" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="27" t="s">
+      <c r="A7" s="30" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="24"/>
-      <c r="C7" s="32">
+      <c r="B7" s="27"/>
+      <c r="C7" s="34">
         <f>IFERROR(VLOOKUP(C4, '🏷️ Catálogo Productos'!A:F, 6, FALSE), 0)</f>
         <v>55000</v>
       </c>
-      <c r="D7" s="24"/>
+      <c r="D7" s="27"/>
     </row>
     <row r="8" spans="1:9" ht="22" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="27" t="s">
+      <c r="A8" s="30" t="s">
         <v>7</v>
       </c>
-      <c r="B8" s="24"/>
-      <c r="C8" s="30">
+      <c r="B8" s="27"/>
+      <c r="C8" s="29">
         <f>IFERROR(VLOOKUP(C4, '🏷️ Catálogo Productos'!A:J, 10, FALSE), 0)</f>
-        <v>15</v>
-      </c>
-      <c r="D8" s="24"/>
+        <v>2</v>
+      </c>
+      <c r="D8" s="27"/>
     </row>
     <row r="9" spans="1:9" ht="22" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="27" t="s">
+      <c r="A9" s="30" t="s">
         <v>8</v>
       </c>
-      <c r="B9" s="24"/>
-      <c r="C9" s="30">
+      <c r="B9" s="27"/>
+      <c r="C9" s="29">
         <f>SUMIF('🛒 Ventas'!C:C, C4, '🛒 Ventas'!F:F)</f>
-        <v>2</v>
-      </c>
-      <c r="D9" s="24"/>
+        <v>0</v>
+      </c>
+      <c r="D9" s="27"/>
     </row>
     <row r="10" spans="1:9" ht="22" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="27" t="s">
+      <c r="A10" s="30" t="s">
         <v>9</v>
       </c>
-      <c r="B10" s="24"/>
-      <c r="C10" s="29" t="str">
+      <c r="B10" s="27"/>
+      <c r="C10" s="36" t="str">
         <f>IF(C4="","", C4 &amp; (SUMIF('🛒 Ventas'!C:C, C4, '🛒 Ventas'!F:F) + 1))</f>
-        <v>TM3</v>
-      </c>
-      <c r="D10" s="24"/>
+        <v>TM1</v>
+      </c>
+      <c r="D10" s="27"/>
     </row>
     <row r="12" spans="1:9" ht="17" x14ac:dyDescent="0.4">
       <c r="A12" s="4" t="s">
@@ -1708,54 +1717,54 @@
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A14" s="26" t="s">
+      <c r="A14" s="28" t="s">
         <v>11</v>
       </c>
-      <c r="B14" s="24"/>
-      <c r="C14" s="26" t="s">
+      <c r="B14" s="27"/>
+      <c r="C14" s="28" t="s">
         <v>12</v>
       </c>
-      <c r="D14" s="24"/>
-      <c r="E14" s="26" t="s">
+      <c r="D14" s="27"/>
+      <c r="E14" s="28" t="s">
         <v>13</v>
       </c>
-      <c r="F14" s="24"/>
-      <c r="G14" s="26" t="s">
+      <c r="F14" s="27"/>
+      <c r="G14" s="28" t="s">
         <v>14</v>
       </c>
-      <c r="H14" s="24"/>
+      <c r="H14" s="27"/>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A15" s="31">
+      <c r="A15" s="33">
         <f>SUM('🏷️ Catálogo Productos'!J4:J14)</f>
-        <v>131</v>
-      </c>
-      <c r="B15" s="24"/>
-      <c r="C15" s="25">
+        <v>14</v>
+      </c>
+      <c r="B15" s="27"/>
+      <c r="C15" s="26">
         <f>SUM('🏷️ Catálogo Productos'!K4:K14)</f>
-        <v>3545000</v>
-      </c>
-      <c r="D15" s="24"/>
-      <c r="E15" s="25">
+        <v>405000</v>
+      </c>
+      <c r="D15" s="27"/>
+      <c r="E15" s="26">
         <f>SUM('🛒 Ventas'!H4:H60)</f>
-        <v>295000</v>
-      </c>
-      <c r="F15" s="24"/>
-      <c r="G15" s="25">
-        <f>SUM('🏢 Activos Fijos'!H4:H12)</f>
-        <v>3100000</v>
-      </c>
-      <c r="H15" s="24"/>
+        <v>0</v>
+      </c>
+      <c r="F15" s="27"/>
+      <c r="G15" s="26">
+        <f>SUM('🏢 Activos Fijos'!H4:H13)</f>
+        <v>4150000</v>
+      </c>
+      <c r="H15" s="27"/>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A16" s="24"/>
-      <c r="B16" s="24"/>
-      <c r="C16" s="24"/>
-      <c r="D16" s="24"/>
-      <c r="E16" s="24"/>
-      <c r="F16" s="24"/>
-      <c r="G16" s="24"/>
-      <c r="H16" s="24"/>
+      <c r="A16" s="27"/>
+      <c r="B16" s="27"/>
+      <c r="C16" s="27"/>
+      <c r="D16" s="27"/>
+      <c r="E16" s="27"/>
+      <c r="F16" s="27"/>
+      <c r="G16" s="27"/>
+      <c r="H16" s="27"/>
     </row>
     <row r="19" spans="1:7" ht="17" x14ac:dyDescent="0.4">
       <c r="A19" s="4" t="s">
@@ -1791,11 +1800,11 @@
       </c>
       <c r="B22" s="7">
         <f>SUMIF('🛒 Ventas'!C:C, "S*", '🛒 Ventas'!F:F)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C22" s="8">
         <f>SUMIF('🛒 Ventas'!C:C, "S*", '🛒 Ventas'!H:H)</f>
-        <v>65000</v>
+        <v>0</v>
       </c>
       <c r="E22" s="6" t="s">
         <v>24</v>
@@ -1806,7 +1815,7 @@
       </c>
       <c r="G22" s="8">
         <f>SUMIF('🛒 Ventas'!I:I, "Nequi", '🛒 Ventas'!H:H)</f>
-        <v>175000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.35">
@@ -1815,11 +1824,11 @@
       </c>
       <c r="B23" s="7">
         <f>SUMIF('🛒 Ventas'!C:C, "P*", '🛒 Ventas'!F:F)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C23" s="8">
         <f>SUMIF('🛒 Ventas'!C:C, "P*", '🛒 Ventas'!H:H)</f>
-        <v>85000</v>
+        <v>0</v>
       </c>
       <c r="E23" s="6" t="s">
         <v>26</v>
@@ -1830,7 +1839,7 @@
       </c>
       <c r="G23" s="8">
         <f>SUMIF('🛒 Ventas'!I:I, "Daviplata", '🛒 Ventas'!H:H)</f>
-        <v>35000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.35">
@@ -1839,11 +1848,11 @@
       </c>
       <c r="B24" s="7">
         <f>SUMIF('🛒 Ventas'!C:C, "T*", '🛒 Ventas'!F:F)</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C24" s="8">
         <f>SUMIF('🛒 Ventas'!C:C, "T*", '🛒 Ventas'!H:H)</f>
-        <v>110000</v>
+        <v>0</v>
       </c>
       <c r="E24" s="6" t="s">
         <v>28</v>
@@ -1854,7 +1863,7 @@
       </c>
       <c r="G24" s="8">
         <f>SUMIF('🛒 Ventas'!I:I, "Efectivo", '🛒 Ventas'!H:H)</f>
-        <v>85000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.35">
@@ -1887,11 +1896,11 @@
       </c>
       <c r="B26" s="7">
         <f>SUMIF('🛒 Ventas'!C:C, "A*", '🛒 Ventas'!F:F)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C26" s="8">
         <f>SUMIF('🛒 Ventas'!C:C, "A*", '🛒 Ventas'!H:H)</f>
-        <v>35000</v>
+        <v>0</v>
       </c>
       <c r="E26" s="6" t="s">
         <v>32</v>
@@ -1911,11 +1920,11 @@
       </c>
       <c r="B27" s="10">
         <f>SUM(B22:B26)</f>
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="C27" s="11">
         <f>SUM(C22:C26)</f>
-        <v>295000</v>
+        <v>0</v>
       </c>
       <c r="E27" s="9" t="s">
         <v>33</v>
@@ -1926,7 +1935,7 @@
       </c>
       <c r="G27" s="11">
         <f>SUM(G22:G26)</f>
-        <v>295000</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -1947,14 +1956,14 @@
     <mergeCell ref="C4:D4"/>
     <mergeCell ref="C10:D10"/>
     <mergeCell ref="A7:B7"/>
+    <mergeCell ref="G15:H16"/>
+    <mergeCell ref="C14:D14"/>
+    <mergeCell ref="E14:F14"/>
     <mergeCell ref="C9:D9"/>
     <mergeCell ref="A4:B4"/>
     <mergeCell ref="C6:D6"/>
     <mergeCell ref="E15:F16"/>
     <mergeCell ref="C5:D5"/>
-    <mergeCell ref="G15:H16"/>
-    <mergeCell ref="C14:D14"/>
-    <mergeCell ref="E14:F14"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing r:id="rId1"/>
@@ -2118,20 +2127,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="40" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="34" t="s">
+      <c r="A1" s="24" t="s">
         <v>55</v>
       </c>
-      <c r="B1" s="35"/>
-      <c r="C1" s="35"/>
-      <c r="D1" s="35"/>
-      <c r="E1" s="35"/>
-      <c r="F1" s="35"/>
-      <c r="G1" s="35"/>
-      <c r="H1" s="35"/>
-      <c r="I1" s="35"/>
-      <c r="J1" s="35"/>
-      <c r="K1" s="35"/>
-      <c r="L1" s="35"/>
+      <c r="B1" s="25"/>
+      <c r="C1" s="25"/>
+      <c r="D1" s="25"/>
+      <c r="E1" s="25"/>
+      <c r="F1" s="25"/>
+      <c r="G1" s="25"/>
+      <c r="H1" s="25"/>
+      <c r="I1" s="25"/>
+      <c r="J1" s="25"/>
+      <c r="K1" s="25"/>
+      <c r="L1" s="25"/>
     </row>
     <row r="3" spans="1:12" ht="28" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="14" t="s">
@@ -2191,27 +2200,27 @@
         <v>55000</v>
       </c>
       <c r="G4" s="7">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="H4" s="7">
         <f>SUMIF('📥 Entradas'!C:C, A4, '📥 Entradas'!F:F)</f>
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="I4" s="7">
         <f>SUMIF('🛒 Ventas'!C:C, A4, '🛒 Ventas'!F:F)</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J4" s="3">
         <f t="shared" ref="J4:J14" si="0">G4+H4-I4</f>
-        <v>15</v>
+        <v>2</v>
       </c>
       <c r="K4" s="8">
         <f t="shared" ref="K4:K14" si="1">J4*E4</f>
-        <v>375000</v>
+        <v>50000</v>
       </c>
       <c r="L4" s="15" t="str">
         <f t="shared" ref="L4:L14" si="2">IF(J4&lt;=0, "❌ Agotado", IF(J4&lt;=3, "⚠️ Stock Bajo", "✅ Disponible"))</f>
-        <v>✅ Disponible</v>
+        <v>⚠️ Stock Bajo</v>
       </c>
     </row>
     <row r="5" spans="1:12" ht="20" customHeight="1" x14ac:dyDescent="0.35">
@@ -2233,8 +2242,8 @@
       <c r="F5" s="18">
         <v>55000</v>
       </c>
-      <c r="G5" s="19">
-        <v>10</v>
+      <c r="G5" s="7">
+        <v>1</v>
       </c>
       <c r="H5" s="19">
         <f>SUMIF('📥 Entradas'!C:C, A5, '📥 Entradas'!F:F)</f>
@@ -2246,15 +2255,15 @@
       </c>
       <c r="J5" s="20">
         <f t="shared" si="0"/>
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="K5" s="18">
         <f t="shared" si="1"/>
-        <v>250000</v>
+        <v>25000</v>
       </c>
       <c r="L5" s="16" t="str">
         <f t="shared" si="2"/>
-        <v>✅ Disponible</v>
+        <v>⚠️ Stock Bajo</v>
       </c>
     </row>
     <row r="6" spans="1:12" ht="20" customHeight="1" x14ac:dyDescent="0.35">
@@ -2277,7 +2286,7 @@
         <v>55000</v>
       </c>
       <c r="G6" s="7">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="H6" s="7">
         <f>SUMIF('📥 Entradas'!C:C, A6, '📥 Entradas'!F:F)</f>
@@ -2289,15 +2298,15 @@
       </c>
       <c r="J6" s="3">
         <f t="shared" si="0"/>
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="K6" s="8">
         <f t="shared" si="1"/>
-        <v>200000</v>
+        <v>25000</v>
       </c>
       <c r="L6" s="15" t="str">
         <f t="shared" si="2"/>
-        <v>✅ Disponible</v>
+        <v>⚠️ Stock Bajo</v>
       </c>
     </row>
     <row r="7" spans="1:12" ht="20" customHeight="1" x14ac:dyDescent="0.35">
@@ -2319,28 +2328,28 @@
       <c r="F7" s="18">
         <v>65000</v>
       </c>
-      <c r="G7" s="19">
-        <v>15</v>
+      <c r="G7" s="7">
+        <v>1</v>
       </c>
       <c r="H7" s="19">
         <f>SUMIF('📥 Entradas'!C:C, A7, '📥 Entradas'!F:F)</f>
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="I7" s="19">
         <f>SUMIF('🛒 Ventas'!C:C, A7, '🛒 Ventas'!F:F)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J7" s="20">
         <f t="shared" si="0"/>
-        <v>19</v>
+        <v>2</v>
       </c>
       <c r="K7" s="18">
         <f t="shared" si="1"/>
-        <v>570000</v>
+        <v>60000</v>
       </c>
       <c r="L7" s="16" t="str">
         <f t="shared" si="2"/>
-        <v>✅ Disponible</v>
+        <v>⚠️ Stock Bajo</v>
       </c>
     </row>
     <row r="8" spans="1:12" ht="20" customHeight="1" x14ac:dyDescent="0.35">
@@ -2363,7 +2372,7 @@
         <v>65000</v>
       </c>
       <c r="G8" s="7">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="H8" s="7">
         <f>SUMIF('📥 Entradas'!C:C, A8, '📥 Entradas'!F:F)</f>
@@ -2375,15 +2384,15 @@
       </c>
       <c r="J8" s="3">
         <f t="shared" si="0"/>
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="K8" s="8">
         <f t="shared" si="1"/>
-        <v>450000</v>
+        <v>30000</v>
       </c>
       <c r="L8" s="15" t="str">
         <f t="shared" si="2"/>
-        <v>✅ Disponible</v>
+        <v>⚠️ Stock Bajo</v>
       </c>
     </row>
     <row r="9" spans="1:12" ht="20" customHeight="1" x14ac:dyDescent="0.35">
@@ -2405,8 +2414,8 @@
       <c r="F9" s="18">
         <v>65000</v>
       </c>
-      <c r="G9" s="19">
-        <v>10</v>
+      <c r="G9" s="7">
+        <v>1</v>
       </c>
       <c r="H9" s="19">
         <f>SUMIF('📥 Entradas'!C:C, A9, '📥 Entradas'!F:F)</f>
@@ -2418,15 +2427,15 @@
       </c>
       <c r="J9" s="20">
         <f t="shared" si="0"/>
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="K9" s="18">
         <f t="shared" si="1"/>
-        <v>300000</v>
+        <v>30000</v>
       </c>
       <c r="L9" s="16" t="str">
         <f t="shared" si="2"/>
-        <v>✅ Disponible</v>
+        <v>⚠️ Stock Bajo</v>
       </c>
     </row>
     <row r="10" spans="1:12" ht="20" customHeight="1" x14ac:dyDescent="0.35">
@@ -2449,7 +2458,7 @@
         <v>85000</v>
       </c>
       <c r="G10" s="7">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="H10" s="7">
         <f>SUMIF('📥 Entradas'!C:C, A10, '📥 Entradas'!F:F)</f>
@@ -2457,19 +2466,19 @@
       </c>
       <c r="I10" s="7">
         <f>SUMIF('🛒 Ventas'!C:C, A10, '🛒 Ventas'!F:F)</f>
+        <v>0</v>
+      </c>
+      <c r="J10" s="3">
+        <f t="shared" si="0"/>
         <v>1</v>
-      </c>
-      <c r="J10" s="3">
-        <f t="shared" si="0"/>
-        <v>5</v>
       </c>
       <c r="K10" s="8">
         <f t="shared" si="1"/>
-        <v>200000</v>
+        <v>40000</v>
       </c>
       <c r="L10" s="15" t="str">
         <f t="shared" si="2"/>
-        <v>✅ Disponible</v>
+        <v>⚠️ Stock Bajo</v>
       </c>
     </row>
     <row r="11" spans="1:12" ht="20" customHeight="1" x14ac:dyDescent="0.35">
@@ -2491,8 +2500,8 @@
       <c r="F11" s="18">
         <v>85000</v>
       </c>
-      <c r="G11" s="19">
-        <v>8</v>
+      <c r="G11" s="7">
+        <v>1</v>
       </c>
       <c r="H11" s="19">
         <f>SUMIF('📥 Entradas'!C:C, A11, '📥 Entradas'!F:F)</f>
@@ -2504,15 +2513,15 @@
       </c>
       <c r="J11" s="20">
         <f t="shared" si="0"/>
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="K11" s="18">
         <f t="shared" si="1"/>
-        <v>320000</v>
+        <v>40000</v>
       </c>
       <c r="L11" s="16" t="str">
         <f t="shared" si="2"/>
-        <v>✅ Disponible</v>
+        <v>⚠️ Stock Bajo</v>
       </c>
     </row>
     <row r="12" spans="1:12" ht="20" customHeight="1" x14ac:dyDescent="0.35">
@@ -2535,7 +2544,7 @@
         <v>85000</v>
       </c>
       <c r="G12" s="7">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="H12" s="7">
         <f>SUMIF('📥 Entradas'!C:C, A12, '📥 Entradas'!F:F)</f>
@@ -2547,15 +2556,15 @@
       </c>
       <c r="J12" s="3">
         <f t="shared" si="0"/>
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="K12" s="8">
         <f t="shared" si="1"/>
-        <v>200000</v>
+        <v>40000</v>
       </c>
       <c r="L12" s="15" t="str">
         <f t="shared" si="2"/>
-        <v>✅ Disponible</v>
+        <v>⚠️ Stock Bajo</v>
       </c>
     </row>
     <row r="13" spans="1:12" ht="20" customHeight="1" x14ac:dyDescent="0.35">
@@ -2577,8 +2586,8 @@
       <c r="F13" s="18">
         <v>75000</v>
       </c>
-      <c r="G13" s="19">
-        <v>7</v>
+      <c r="G13" s="7">
+        <v>1</v>
       </c>
       <c r="H13" s="19">
         <f>SUMIF('📥 Entradas'!C:C, A13, '📥 Entradas'!F:F)</f>
@@ -2590,15 +2599,15 @@
       </c>
       <c r="J13" s="20">
         <f t="shared" si="0"/>
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="K13" s="18">
         <f t="shared" si="1"/>
-        <v>245000</v>
+        <v>35000</v>
       </c>
       <c r="L13" s="16" t="str">
         <f t="shared" si="2"/>
-        <v>✅ Disponible</v>
+        <v>⚠️ Stock Bajo</v>
       </c>
     </row>
     <row r="14" spans="1:12" ht="20" customHeight="1" x14ac:dyDescent="0.35">
@@ -2621,27 +2630,27 @@
         <v>35000</v>
       </c>
       <c r="G14" s="7">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="H14" s="7">
         <f>SUMIF('📥 Entradas'!C:C, A14, '📥 Entradas'!F:F)</f>
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="I14" s="7">
         <f>SUMIF('🛒 Ventas'!C:C, A14, '🛒 Ventas'!F:F)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J14" s="3">
         <f t="shared" si="0"/>
-        <v>29</v>
+        <v>2</v>
       </c>
       <c r="K14" s="8">
         <f t="shared" si="1"/>
-        <v>435000</v>
+        <v>30000</v>
       </c>
       <c r="L14" s="15" t="str">
         <f t="shared" si="2"/>
-        <v>✅ Disponible</v>
+        <v>⚠️ Stock Bajo</v>
       </c>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.35">
@@ -2653,25 +2662,22 @@
       <c r="D15" s="9"/>
       <c r="E15" s="9"/>
       <c r="F15" s="9"/>
-      <c r="G15" s="10">
-        <f>SUM(G4:G14)</f>
-        <v>116</v>
-      </c>
+      <c r="G15" s="10"/>
       <c r="H15" s="10">
         <f>SUM(H4:H14)</f>
-        <v>20</v>
+        <v>3</v>
       </c>
       <c r="I15" s="10">
         <f>SUM(I4:I14)</f>
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="J15" s="10">
         <f>SUM(J4:J14)</f>
-        <v>131</v>
+        <v>14</v>
       </c>
       <c r="K15" s="11">
         <f>SUM(K4:K14)</f>
-        <v>3545000</v>
+        <v>405000</v>
       </c>
       <c r="L15" s="9"/>
     </row>
@@ -2698,17 +2704,17 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="40" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="34" t="s">
+      <c r="A1" s="24" t="s">
         <v>83</v>
       </c>
-      <c r="B1" s="35"/>
-      <c r="C1" s="35"/>
-      <c r="D1" s="35"/>
-      <c r="E1" s="35"/>
-      <c r="F1" s="35"/>
-      <c r="G1" s="35"/>
-      <c r="H1" s="35"/>
-      <c r="I1" s="35"/>
+      <c r="B1" s="25"/>
+      <c r="C1" s="25"/>
+      <c r="D1" s="25"/>
+      <c r="E1" s="25"/>
+      <c r="F1" s="25"/>
+      <c r="G1" s="25"/>
+      <c r="H1" s="25"/>
+      <c r="I1" s="25"/>
     </row>
     <row r="3" spans="1:9" ht="28" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="14" t="s">
@@ -2758,7 +2764,7 @@
         <v>M</v>
       </c>
       <c r="F4" s="7">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G4" s="8">
         <f>IFERROR(VLOOKUP(C4, '🏷️ Catálogo Productos'!A:E, 5, FALSE), 0)</f>
@@ -2766,7 +2772,7 @@
       </c>
       <c r="H4" s="8">
         <f>F4*G4</f>
-        <v>125000</v>
+        <v>25000</v>
       </c>
       <c r="I4" s="6" t="s">
         <v>93</v>
@@ -2791,7 +2797,7 @@
         <v>M</v>
       </c>
       <c r="F5" s="7">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G5" s="8">
         <f>IFERROR(VLOOKUP(C5, '🏷️ Catálogo Productos'!A:E, 5, FALSE), 0)</f>
@@ -2799,7 +2805,7 @@
       </c>
       <c r="H5" s="8">
         <f>F5*G5</f>
-        <v>150000</v>
+        <v>30000</v>
       </c>
       <c r="I5" s="6" t="s">
         <v>93</v>
@@ -2824,7 +2830,7 @@
         <v>Única</v>
       </c>
       <c r="F6" s="7">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="G6" s="8">
         <f>IFERROR(VLOOKUP(C6, '🏷️ Catálogo Productos'!A:E, 5, FALSE), 0)</f>
@@ -2832,7 +2838,7 @@
       </c>
       <c r="H6" s="8">
         <f>F6*G6</f>
-        <v>150000</v>
+        <v>15000</v>
       </c>
       <c r="I6" s="6" t="s">
         <v>97</v>
@@ -3450,18 +3456,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="40" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="34" t="s">
+      <c r="A1" s="24" t="s">
         <v>121</v>
       </c>
-      <c r="B1" s="35"/>
-      <c r="C1" s="35"/>
-      <c r="D1" s="35"/>
-      <c r="E1" s="35"/>
-      <c r="F1" s="35"/>
-      <c r="G1" s="35"/>
-      <c r="H1" s="35"/>
-      <c r="I1" s="35"/>
-      <c r="J1" s="35"/>
+      <c r="B1" s="25"/>
+      <c r="C1" s="25"/>
+      <c r="D1" s="25"/>
+      <c r="E1" s="25"/>
+      <c r="F1" s="25"/>
+      <c r="G1" s="25"/>
+      <c r="H1" s="25"/>
+      <c r="I1" s="25"/>
+      <c r="J1" s="25"/>
     </row>
     <row r="3" spans="1:10" ht="28" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="14" t="s">
@@ -3514,16 +3520,14 @@
         <f>IFERROR(VLOOKUP(C4, '🏷️ Catálogo Productos'!A:D, 4, FALSE), "")</f>
         <v>M</v>
       </c>
-      <c r="F4" s="7">
-        <v>1</v>
-      </c>
+      <c r="F4" s="7"/>
       <c r="G4" s="8">
         <f>IFERROR(VLOOKUP(C4, '🏷️ Catálogo Productos'!A:F, 6, FALSE), 0)</f>
         <v>55000</v>
       </c>
       <c r="H4" s="8">
         <f>F4*G4</f>
-        <v>55000</v>
+        <v>0</v>
       </c>
       <c r="I4" s="15" t="s">
         <v>24</v>
@@ -3551,16 +3555,14 @@
         <f>IFERROR(VLOOKUP(C5, '🏷️ Catálogo Productos'!A:D, 4, FALSE), "")</f>
         <v>M</v>
       </c>
-      <c r="F5" s="7">
-        <v>1</v>
-      </c>
+      <c r="F5" s="7"/>
       <c r="G5" s="8">
         <f>IFERROR(VLOOKUP(C5, '🏷️ Catálogo Productos'!A:F, 6, FALSE), 0)</f>
         <v>65000</v>
       </c>
       <c r="H5" s="8">
         <f>F5*G5</f>
-        <v>65000</v>
+        <v>0</v>
       </c>
       <c r="I5" s="15" t="s">
         <v>24</v>
@@ -3588,16 +3590,14 @@
         <f>IFERROR(VLOOKUP(C6, '🏷️ Catálogo Productos'!A:D, 4, FALSE), "")</f>
         <v>S</v>
       </c>
-      <c r="F6" s="7">
-        <v>1</v>
-      </c>
+      <c r="F6" s="7"/>
       <c r="G6" s="8">
         <f>IFERROR(VLOOKUP(C6, '🏷️ Catálogo Productos'!A:F, 6, FALSE), 0)</f>
         <v>85000</v>
       </c>
       <c r="H6" s="8">
         <f>F6*G6</f>
-        <v>85000</v>
+        <v>0</v>
       </c>
       <c r="I6" s="15" t="s">
         <v>28</v>
@@ -3625,16 +3625,14 @@
         <f>IFERROR(VLOOKUP(C7, '🏷️ Catálogo Productos'!A:D, 4, FALSE), "")</f>
         <v>Única</v>
       </c>
-      <c r="F7" s="7">
-        <v>1</v>
-      </c>
+      <c r="F7" s="7"/>
       <c r="G7" s="8">
         <f>IFERROR(VLOOKUP(C7, '🏷️ Catálogo Productos'!A:F, 6, FALSE), 0)</f>
         <v>35000</v>
       </c>
       <c r="H7" s="8">
         <f>F7*G7</f>
-        <v>35000</v>
+        <v>0</v>
       </c>
       <c r="I7" s="15" t="s">
         <v>26</v>
@@ -3662,16 +3660,14 @@
         <f>IFERROR(VLOOKUP(C8, '🏷️ Catálogo Productos'!A:D, 4, FALSE), "")</f>
         <v>M</v>
       </c>
-      <c r="F8" s="7">
-        <v>1</v>
-      </c>
+      <c r="F8" s="7"/>
       <c r="G8" s="8">
         <f>IFERROR(VLOOKUP(C8, '🏷️ Catálogo Productos'!A:F, 6, FALSE), 0)</f>
         <v>55000</v>
       </c>
       <c r="H8" s="8">
         <f>F8*G8</f>
-        <v>55000</v>
+        <v>0</v>
       </c>
       <c r="I8" s="15" t="s">
         <v>24</v>
@@ -4565,7 +4561,7 @@
         <v/>
       </c>
       <c r="H41" s="22" t="str">
-        <f t="shared" ref="H41:H72" si="1">IF(F41="","",F41*G41)</f>
+        <f t="shared" ref="H41:H59" si="1">IF(F41="","",F41*G41)</f>
         <v/>
       </c>
       <c r="I41" s="1"/>
@@ -5089,7 +5085,7 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="17" customWidth="1"/>
-    <col min="2" max="2" width="37.54296875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="40.81640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="24" customWidth="1"/>
     <col min="4" max="4" width="23" customWidth="1"/>
     <col min="5" max="5" width="18" customWidth="1"/>
@@ -5101,18 +5097,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="40" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="34" t="s">
+      <c r="A1" s="24" t="s">
         <v>134</v>
       </c>
-      <c r="B1" s="35"/>
-      <c r="C1" s="35"/>
-      <c r="D1" s="35"/>
-      <c r="E1" s="35"/>
-      <c r="F1" s="35"/>
-      <c r="G1" s="35"/>
-      <c r="H1" s="35"/>
-      <c r="I1" s="35"/>
-      <c r="J1" s="35"/>
+      <c r="B1" s="25"/>
+      <c r="C1" s="25"/>
+      <c r="D1" s="25"/>
+      <c r="E1" s="25"/>
+      <c r="F1" s="25"/>
+      <c r="G1" s="25"/>
+      <c r="H1" s="25"/>
+      <c r="I1" s="25"/>
+      <c r="J1" s="25"/>
     </row>
     <row r="3" spans="1:10" ht="28" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="14" t="s">
@@ -5151,7 +5147,7 @@
         <v>145</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="C4" s="6" t="s">
         <v>42</v>
@@ -5169,7 +5165,7 @@
         <v>1200000</v>
       </c>
       <c r="H4" s="8">
-        <f t="shared" ref="H4:H10" si="0">E4*G4</f>
+        <f t="shared" ref="H4:H5" si="0">E4*G4</f>
         <v>2400000</v>
       </c>
       <c r="I4" s="15" t="s">
@@ -5183,8 +5179,8 @@
       <c r="A5" s="16" t="s">
         <v>149</v>
       </c>
-      <c r="B5" s="17" t="s">
-        <v>194</v>
+      <c r="B5" s="6" t="s">
+        <v>195</v>
       </c>
       <c r="C5" s="17" t="s">
         <v>42</v>
@@ -5193,7 +5189,7 @@
         <v>146</v>
       </c>
       <c r="E5" s="19">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F5" s="15" t="s">
         <v>41</v>
@@ -5203,7 +5199,7 @@
       </c>
       <c r="H5" s="18">
         <f t="shared" si="0"/>
-        <v>350000</v>
+        <v>1050000</v>
       </c>
       <c r="I5" s="16" t="s">
         <v>147</v>
@@ -5217,7 +5213,7 @@
         <v>151</v>
       </c>
       <c r="B6" s="17" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="C6" s="17" t="s">
         <v>42</v>
@@ -5249,205 +5245,224 @@
       <c r="A7" s="16" t="s">
         <v>156</v>
       </c>
-      <c r="B7" s="6" t="s">
-        <v>152</v>
-      </c>
-      <c r="C7" s="6" t="s">
-        <v>45</v>
-      </c>
-      <c r="D7" s="6" t="s">
-        <v>153</v>
-      </c>
-      <c r="E7" s="7"/>
+      <c r="B7" s="17" t="s">
+        <v>197</v>
+      </c>
+      <c r="C7" s="17" t="s">
+        <v>42</v>
+      </c>
+      <c r="D7" s="17" t="s">
+        <v>146</v>
+      </c>
+      <c r="E7" s="19">
+        <v>1</v>
+      </c>
       <c r="F7" s="15" t="s">
         <v>41</v>
       </c>
-      <c r="G7" s="8">
-        <v>15000</v>
-      </c>
-      <c r="H7" s="8">
-        <f>E7*G7</f>
-        <v>0</v>
-      </c>
-      <c r="I7" s="15" t="s">
-        <v>154</v>
-      </c>
-      <c r="J7" s="6" t="s">
-        <v>155</v>
+      <c r="G7" s="18">
+        <v>350000</v>
+      </c>
+      <c r="H7" s="18">
+        <f t="shared" ref="H7" si="2">E7*G7</f>
+        <v>350000</v>
+      </c>
+      <c r="I7" s="16" t="s">
+        <v>147</v>
+      </c>
+      <c r="J7" s="17" t="s">
+        <v>196</v>
       </c>
     </row>
     <row r="8" spans="1:10" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="15" t="s">
         <v>161</v>
       </c>
-      <c r="B8" s="17" t="s">
-        <v>157</v>
-      </c>
-      <c r="C8" s="17" t="s">
-        <v>48</v>
-      </c>
-      <c r="D8" s="17" t="s">
-        <v>158</v>
-      </c>
-      <c r="E8" s="19"/>
+      <c r="B8" s="6" t="s">
+        <v>152</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="D8" s="6" t="s">
+        <v>153</v>
+      </c>
+      <c r="E8" s="7"/>
       <c r="F8" s="15" t="s">
         <v>41</v>
       </c>
-      <c r="G8" s="18">
-        <v>45000</v>
-      </c>
-      <c r="H8" s="18">
-        <f>E8*G8</f>
+      <c r="G8" s="8">
+        <v>15000</v>
+      </c>
+      <c r="H8" s="8">
+        <f t="shared" ref="H8:H13" si="3">E8*G8</f>
         <v>0</v>
       </c>
-      <c r="I8" s="16" t="s">
-        <v>159</v>
-      </c>
-      <c r="J8" s="17" t="s">
-        <v>160</v>
+      <c r="I8" s="15" t="s">
+        <v>154</v>
+      </c>
+      <c r="J8" s="6" t="s">
+        <v>155</v>
       </c>
     </row>
     <row r="9" spans="1:10" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="16" t="s">
         <v>165</v>
       </c>
-      <c r="B9" s="6" t="s">
-        <v>162</v>
-      </c>
-      <c r="C9" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="D9" s="6" t="s">
-        <v>146</v>
-      </c>
-      <c r="E9" s="7"/>
+      <c r="B9" s="17" t="s">
+        <v>157</v>
+      </c>
+      <c r="C9" s="17" t="s">
+        <v>48</v>
+      </c>
+      <c r="D9" s="17" t="s">
+        <v>158</v>
+      </c>
+      <c r="E9" s="19"/>
       <c r="F9" s="15" t="s">
         <v>41</v>
       </c>
-      <c r="G9" s="8">
-        <v>60000</v>
-      </c>
-      <c r="H9" s="8">
-        <f>E9*G9</f>
+      <c r="G9" s="18">
+        <v>45000</v>
+      </c>
+      <c r="H9" s="18">
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="I9" s="15" t="s">
-        <v>163</v>
-      </c>
-      <c r="J9" s="6" t="s">
-        <v>164</v>
+      <c r="I9" s="16" t="s">
+        <v>159</v>
+      </c>
+      <c r="J9" s="17" t="s">
+        <v>160</v>
       </c>
     </row>
     <row r="10" spans="1:10" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="15" t="s">
         <v>169</v>
       </c>
-      <c r="B10" s="17" t="s">
-        <v>166</v>
-      </c>
-      <c r="C10" s="17" t="s">
-        <v>48</v>
-      </c>
-      <c r="D10" s="17" t="s">
-        <v>132</v>
-      </c>
-      <c r="E10" s="19"/>
+      <c r="B10" s="6" t="s">
+        <v>162</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="D10" s="6" t="s">
+        <v>146</v>
+      </c>
+      <c r="E10" s="7"/>
       <c r="F10" s="15" t="s">
         <v>41</v>
       </c>
-      <c r="G10" s="18">
-        <v>450000</v>
-      </c>
-      <c r="H10" s="18">
-        <f>E10*G10</f>
+      <c r="G10" s="8">
+        <v>60000</v>
+      </c>
+      <c r="H10" s="8">
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="I10" s="16" t="s">
-        <v>167</v>
-      </c>
-      <c r="J10" s="17" t="s">
-        <v>168</v>
+      <c r="I10" s="15" t="s">
+        <v>163</v>
+      </c>
+      <c r="J10" s="6" t="s">
+        <v>164</v>
       </c>
     </row>
     <row r="11" spans="1:10" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="16" t="s">
         <v>174</v>
       </c>
-      <c r="B11" s="6" t="s">
-        <v>170</v>
-      </c>
-      <c r="C11" s="6" t="s">
-        <v>51</v>
-      </c>
-      <c r="D11" s="6" t="s">
-        <v>171</v>
-      </c>
-      <c r="E11" s="7"/>
+      <c r="B11" s="17" t="s">
+        <v>166</v>
+      </c>
+      <c r="C11" s="17" t="s">
+        <v>48</v>
+      </c>
+      <c r="D11" s="17" t="s">
+        <v>132</v>
+      </c>
+      <c r="E11" s="19"/>
       <c r="F11" s="15" t="s">
         <v>41</v>
       </c>
-      <c r="G11" s="8">
-        <v>80000</v>
-      </c>
-      <c r="H11" s="8">
-        <f>E11*G11</f>
+      <c r="G11" s="18">
+        <v>450000</v>
+      </c>
+      <c r="H11" s="18">
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="I11" s="15" t="s">
-        <v>172</v>
-      </c>
-      <c r="J11" s="6" t="s">
-        <v>173</v>
+      <c r="I11" s="16" t="s">
+        <v>167</v>
+      </c>
+      <c r="J11" s="17" t="s">
+        <v>168</v>
       </c>
     </row>
     <row r="12" spans="1:10" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="16" t="s">
-        <v>195</v>
-      </c>
-      <c r="B12" s="17" t="s">
-        <v>175</v>
-      </c>
-      <c r="C12" s="17" t="s">
-        <v>53</v>
-      </c>
-      <c r="D12" s="17" t="s">
-        <v>146</v>
-      </c>
-      <c r="E12" s="19"/>
+        <v>194</v>
+      </c>
+      <c r="B12" s="6" t="s">
+        <v>170</v>
+      </c>
+      <c r="C12" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="D12" s="6" t="s">
+        <v>171</v>
+      </c>
+      <c r="E12" s="7"/>
       <c r="F12" s="15" t="s">
         <v>41</v>
       </c>
-      <c r="G12" s="18">
-        <v>850000</v>
-      </c>
-      <c r="H12" s="18">
-        <f>E12*G12</f>
+      <c r="G12" s="8">
+        <v>80000</v>
+      </c>
+      <c r="H12" s="8">
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="I12" s="16" t="s">
-        <v>176</v>
-      </c>
-      <c r="J12" s="17" t="s">
-        <v>177</v>
+      <c r="I12" s="15" t="s">
+        <v>172</v>
+      </c>
+      <c r="J12" s="6" t="s">
+        <v>173</v>
       </c>
     </row>
     <row r="13" spans="1:10" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="15" t="s">
-        <v>179</v>
-      </c>
-      <c r="B13" s="17"/>
-      <c r="C13" s="17"/>
-      <c r="D13" s="17"/>
+        <v>178</v>
+      </c>
+      <c r="B13" s="17" t="s">
+        <v>198</v>
+      </c>
+      <c r="C13" s="17" t="s">
+        <v>53</v>
+      </c>
+      <c r="D13" s="17" t="s">
+        <v>146</v>
+      </c>
       <c r="E13" s="19"/>
-      <c r="F13" s="16"/>
-      <c r="G13" s="18"/>
-      <c r="H13" s="18"/>
-      <c r="I13" s="16"/>
-      <c r="J13" s="36"/>
+      <c r="F13" s="15" t="s">
+        <v>41</v>
+      </c>
+      <c r="G13" s="18">
+        <v>850000</v>
+      </c>
+      <c r="H13" s="18">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="I13" s="16" t="s">
+        <v>175</v>
+      </c>
+      <c r="J13" s="17" t="s">
+        <v>176</v>
+      </c>
     </row>
     <row r="14" spans="1:10" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="15" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="B14" s="17"/>
       <c r="C14" s="17"/>
@@ -5457,11 +5472,11 @@
       <c r="G14" s="18"/>
       <c r="H14" s="18"/>
       <c r="I14" s="16"/>
-      <c r="J14" s="36"/>
+      <c r="J14" s="23"/>
     </row>
     <row r="15" spans="1:10" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="15" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="B15" s="17"/>
       <c r="C15" s="17"/>
@@ -5471,11 +5486,11 @@
       <c r="G15" s="18"/>
       <c r="H15" s="18"/>
       <c r="I15" s="16"/>
-      <c r="J15" s="36"/>
+      <c r="J15" s="23"/>
     </row>
     <row r="16" spans="1:10" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="15" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="B16" s="17"/>
       <c r="C16" s="17"/>
@@ -5485,11 +5500,11 @@
       <c r="G16" s="18"/>
       <c r="H16" s="18"/>
       <c r="I16" s="16"/>
-      <c r="J16" s="36"/>
+      <c r="J16" s="23"/>
     </row>
     <row r="17" spans="1:10" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="15" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="B17" s="17"/>
       <c r="C17" s="17"/>
@@ -5499,11 +5514,11 @@
       <c r="G17" s="18"/>
       <c r="H17" s="18"/>
       <c r="I17" s="16"/>
-      <c r="J17" s="36"/>
+      <c r="J17" s="23"/>
     </row>
     <row r="18" spans="1:10" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="15" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="B18" s="17"/>
       <c r="C18" s="17"/>
@@ -5513,11 +5528,11 @@
       <c r="G18" s="18"/>
       <c r="H18" s="18"/>
       <c r="I18" s="16"/>
-      <c r="J18" s="36"/>
+      <c r="J18" s="23"/>
     </row>
     <row r="19" spans="1:10" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" s="15" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="B19" s="17"/>
       <c r="C19" s="17"/>
@@ -5527,11 +5542,11 @@
       <c r="G19" s="18"/>
       <c r="H19" s="18"/>
       <c r="I19" s="16"/>
-      <c r="J19" s="36"/>
+      <c r="J19" s="23"/>
     </row>
     <row r="20" spans="1:10" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20" s="15" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="B20" s="17"/>
       <c r="C20" s="17"/>
@@ -5541,11 +5556,11 @@
       <c r="G20" s="18"/>
       <c r="H20" s="18"/>
       <c r="I20" s="16"/>
-      <c r="J20" s="36"/>
+      <c r="J20" s="23"/>
     </row>
     <row r="21" spans="1:10" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A21" s="15" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="B21" s="17"/>
       <c r="C21" s="17"/>
@@ -5558,35 +5573,35 @@
     </row>
     <row r="22" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A22" s="15" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="J22" s="9"/>
     </row>
     <row r="23" spans="1:10" ht="20" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A23" s="15" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B23" s="9"/>
       <c r="C23" s="9"/>
       <c r="D23" s="21" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="E23" s="10">
-        <f>SUM(E4:E12)</f>
-        <v>4</v>
+        <f>SUM(E4:E13)</f>
+        <v>7</v>
       </c>
       <c r="F23" s="9"/>
       <c r="G23" s="9"/>
       <c r="H23" s="11">
-        <f>SUM(H4:H12)</f>
-        <v>3100000</v>
+        <f>SUM(H4:H13)</f>
+        <v>4150000</v>
       </c>
       <c r="I23" s="9"/>
       <c r="J23" s="1"/>
     </row>
     <row r="24" spans="1:10" ht="20" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A24" s="15" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="B24" s="1"/>
       <c r="C24" s="1"/>
@@ -5595,7 +5610,7 @@
       <c r="F24" s="1"/>
       <c r="G24" s="1"/>
       <c r="H24" s="22" t="str">
-        <f t="shared" ref="H24:H37" si="2">IF(E24="","",E24*G24)</f>
+        <f t="shared" ref="H24:H37" si="4">IF(E24="","",E24*G24)</f>
         <v/>
       </c>
       <c r="I24" s="1"/>
@@ -5603,7 +5618,7 @@
     </row>
     <row r="25" spans="1:10" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A25" s="15" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="B25" s="1"/>
       <c r="C25" s="1"/>
@@ -5612,7 +5627,7 @@
       <c r="F25" s="1"/>
       <c r="G25" s="1"/>
       <c r="H25" s="22" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="I25" s="1"/>
@@ -5620,7 +5635,7 @@
     </row>
     <row r="26" spans="1:10" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A26" s="15" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="B26" s="1"/>
       <c r="C26" s="1"/>
@@ -5629,7 +5644,7 @@
       <c r="F26" s="1"/>
       <c r="G26" s="1"/>
       <c r="H26" s="22" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="I26" s="1"/>
@@ -5637,7 +5652,7 @@
     </row>
     <row r="27" spans="1:10" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A27" s="15" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="B27" s="1"/>
       <c r="C27" s="1"/>
@@ -5646,7 +5661,7 @@
       <c r="F27" s="1"/>
       <c r="G27" s="1"/>
       <c r="H27" s="22" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="I27" s="1"/>
@@ -5654,7 +5669,7 @@
     </row>
     <row r="28" spans="1:10" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A28" s="15" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="B28" s="1"/>
       <c r="C28" s="1"/>
@@ -5663,7 +5678,7 @@
       <c r="F28" s="1"/>
       <c r="G28" s="1"/>
       <c r="H28" s="22" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="I28" s="1"/>
@@ -5671,7 +5686,7 @@
     </row>
     <row r="29" spans="1:10" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A29" s="15" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="B29" s="1"/>
       <c r="C29" s="1"/>
@@ -5680,7 +5695,7 @@
       <c r="F29" s="1"/>
       <c r="G29" s="1"/>
       <c r="H29" s="22" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="I29" s="1"/>
@@ -5688,7 +5703,7 @@
     </row>
     <row r="30" spans="1:10" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A30" s="15" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="B30" s="1"/>
       <c r="C30" s="1"/>
@@ -5697,7 +5712,7 @@
       <c r="F30" s="1"/>
       <c r="G30" s="1"/>
       <c r="H30" s="22" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="I30" s="1"/>
@@ -5705,7 +5720,7 @@
     </row>
     <row r="31" spans="1:10" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A31" s="15" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="B31" s="1"/>
       <c r="C31" s="1"/>
@@ -5714,7 +5729,7 @@
       <c r="F31" s="1"/>
       <c r="G31" s="1"/>
       <c r="H31" s="22" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="I31" s="1"/>
@@ -5722,7 +5737,7 @@
     </row>
     <row r="32" spans="1:10" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A32" s="15" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="B32" s="1"/>
       <c r="C32" s="1"/>
@@ -5731,7 +5746,7 @@
       <c r="F32" s="1"/>
       <c r="G32" s="1"/>
       <c r="H32" s="22" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="I32" s="1"/>
@@ -5739,7 +5754,7 @@
     </row>
     <row r="33" spans="1:10" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A33" s="15" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B33" s="1"/>
       <c r="C33" s="1"/>
@@ -5748,7 +5763,7 @@
       <c r="F33" s="1"/>
       <c r="G33" s="1"/>
       <c r="H33" s="22" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="I33" s="1"/>
@@ -5756,7 +5771,7 @@
     </row>
     <row r="34" spans="1:10" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A34" s="15" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B34" s="1"/>
       <c r="C34" s="1"/>
@@ -5765,7 +5780,7 @@
       <c r="F34" s="1"/>
       <c r="G34" s="1"/>
       <c r="H34" s="22" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="I34" s="1"/>
@@ -5773,7 +5788,7 @@
     </row>
     <row r="35" spans="1:10" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A35" s="15" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="B35" s="1"/>
       <c r="C35" s="1"/>
@@ -5782,7 +5797,7 @@
       <c r="F35" s="1"/>
       <c r="G35" s="1"/>
       <c r="H35" s="22" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="I35" s="1"/>
@@ -5790,7 +5805,7 @@
     </row>
     <row r="36" spans="1:10" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A36" s="15" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="B36" s="1"/>
       <c r="C36" s="1"/>
@@ -5799,7 +5814,7 @@
       <c r="F36" s="1"/>
       <c r="G36" s="1"/>
       <c r="H36" s="22" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="I36" s="1"/>
@@ -5807,7 +5822,7 @@
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A37" s="15" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="B37" s="1"/>
       <c r="C37" s="1"/>
@@ -5816,7 +5831,7 @@
       <c r="F37" s="1"/>
       <c r="G37" s="1"/>
       <c r="H37" s="22" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="I37" s="1"/>

</xml_diff>

<commit_message>
Agregado modulo de consultas rapidas de disponibilidad
</commit_message>
<xml_diff>
--- a/Control_Inventario_Pole_Dance.xlsx
+++ b/Control_Inventario_Pole_Dance.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cenicanaoff365-my.sharepoint.com/personal/iavar3_cenicanaoff365_onmicrosoft_com/Documents/Escritorio/Academia/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="21" documentId="13_ncr:1_{D8F039D2-5B30-42AD-85ED-01D7E78216B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9A9FECFD-AF0B-4891-848D-55B74A6FD964}"/>
+  <xr:revisionPtr revIDLastSave="24" documentId="13_ncr:1_{D8F039D2-5B30-42AD-85ED-01D7E78216B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{ABF19AC0-A734-464B-A63B-8D632686E1F6}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="2" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="302" uniqueCount="195">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="293" uniqueCount="193">
   <si>
     <t>PANEL DE CONTROL E INVENTARIOS - POLE DANCE ACADEMY</t>
   </si>
@@ -563,12 +563,6 @@
   </si>
   <si>
     <t>ACT-010</t>
-  </si>
-  <si>
-    <t>ACT-011</t>
-  </si>
-  <si>
-    <t>ACT-012</t>
   </si>
   <si>
     <t>ACT-013</t>
@@ -780,7 +774,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -834,30 +828,30 @@
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="164" fontId="10" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
     <xf numFmtId="3" fontId="10" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -867,9 +861,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1603,101 +1594,101 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="40" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="24" t="s">
+      <c r="A1" s="30" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="25"/>
-      <c r="C1" s="25"/>
-      <c r="D1" s="25"/>
-      <c r="E1" s="25"/>
-      <c r="F1" s="25"/>
-      <c r="G1" s="25"/>
-      <c r="H1" s="25"/>
-      <c r="I1" s="25"/>
+      <c r="B1" s="31"/>
+      <c r="C1" s="31"/>
+      <c r="D1" s="31"/>
+      <c r="E1" s="31"/>
+      <c r="F1" s="31"/>
+      <c r="G1" s="31"/>
+      <c r="H1" s="31"/>
+      <c r="I1" s="31"/>
     </row>
     <row r="3" spans="1:9" ht="26" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="26" t="s">
+      <c r="A3" s="29" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="27"/>
-      <c r="C3" s="27"/>
-      <c r="D3" s="27"/>
+      <c r="B3" s="24"/>
+      <c r="C3" s="24"/>
+      <c r="D3" s="24"/>
     </row>
     <row r="4" spans="1:9" ht="32" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="28" t="s">
+      <c r="A4" s="27" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="27"/>
+      <c r="B4" s="24"/>
       <c r="C4" s="34" t="s">
         <v>3</v>
       </c>
-      <c r="D4" s="27"/>
+      <c r="D4" s="24"/>
     </row>
     <row r="5" spans="1:9" ht="22" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="28" t="s">
+      <c r="A5" s="27" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="27"/>
-      <c r="C5" s="36" t="str">
+      <c r="B5" s="24"/>
+      <c r="C5" s="28" t="str">
         <f>IFERROR(VLOOKUP(C4, '🏷️ Catálogo Productos'!A:C, 3, FALSE), "⚠️ Código no encontrado")</f>
         <v>Top Velvet Negro</v>
       </c>
-      <c r="D5" s="27"/>
+      <c r="D5" s="24"/>
     </row>
     <row r="6" spans="1:9" ht="22" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="28" t="s">
+      <c r="A6" s="27" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="27"/>
-      <c r="C6" s="36" t="str">
+      <c r="B6" s="24"/>
+      <c r="C6" s="28" t="str">
         <f>IFERROR(VLOOKUP(C4, '🏷️ Catálogo Productos'!A:D, 4, FALSE), "-")</f>
         <v>M</v>
       </c>
-      <c r="D6" s="27"/>
+      <c r="D6" s="24"/>
     </row>
     <row r="7" spans="1:9" ht="22" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="28" t="s">
+      <c r="A7" s="27" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="27"/>
+      <c r="B7" s="24"/>
       <c r="C7" s="33">
         <f>IFERROR(VLOOKUP(C4, '🏷️ Catálogo Productos'!A:F, 6, FALSE), 0)</f>
         <v>55000</v>
       </c>
-      <c r="D7" s="27"/>
+      <c r="D7" s="24"/>
     </row>
     <row r="8" spans="1:9" ht="22" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="28" t="s">
+      <c r="A8" s="27" t="s">
         <v>7</v>
       </c>
-      <c r="B8" s="27"/>
-      <c r="C8" s="32">
+      <c r="B8" s="24"/>
+      <c r="C8" s="26">
         <f>IFERROR(VLOOKUP(C4, '🏷️ Catálogo Productos'!A:J, 10, FALSE), 0)</f>
         <v>2</v>
       </c>
-      <c r="D8" s="27"/>
+      <c r="D8" s="24"/>
     </row>
     <row r="9" spans="1:9" ht="22" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="28" t="s">
+      <c r="A9" s="27" t="s">
         <v>8</v>
       </c>
-      <c r="B9" s="27"/>
-      <c r="C9" s="32">
+      <c r="B9" s="24"/>
+      <c r="C9" s="26">
         <f>SUMIF('🛒 Ventas'!C:C, C4, '🛒 Ventas'!F:F)</f>
         <v>0</v>
       </c>
-      <c r="D9" s="27"/>
+      <c r="D9" s="24"/>
     </row>
     <row r="10" spans="1:9" ht="22" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="28" t="s">
+      <c r="A10" s="27" t="s">
         <v>9</v>
       </c>
-      <c r="B10" s="27"/>
+      <c r="B10" s="24"/>
       <c r="C10" s="35" t="str">
         <f>IF(C4="","", C4 &amp; (SUMIF('🛒 Ventas'!C:C, C4, '🛒 Ventas'!F:F) + 1))</f>
         <v>TM1</v>
       </c>
-      <c r="D10" s="27"/>
+      <c r="D10" s="24"/>
     </row>
     <row r="12" spans="1:9" ht="17" x14ac:dyDescent="0.4">
       <c r="A12" s="4" t="s">
@@ -1705,54 +1696,54 @@
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A14" s="31" t="s">
+      <c r="A14" s="25" t="s">
         <v>11</v>
       </c>
-      <c r="B14" s="27"/>
-      <c r="C14" s="31" t="s">
+      <c r="B14" s="24"/>
+      <c r="C14" s="25" t="s">
         <v>12</v>
       </c>
-      <c r="D14" s="27"/>
-      <c r="E14" s="31" t="s">
+      <c r="D14" s="24"/>
+      <c r="E14" s="25" t="s">
         <v>13</v>
       </c>
-      <c r="F14" s="27"/>
-      <c r="G14" s="31" t="s">
+      <c r="F14" s="24"/>
+      <c r="G14" s="25" t="s">
         <v>14</v>
       </c>
-      <c r="H14" s="27"/>
+      <c r="H14" s="24"/>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A15" s="29">
+      <c r="A15" s="32">
         <f>SUM('🏷️ Catálogo Productos'!J2:J12)</f>
         <v>14</v>
       </c>
-      <c r="B15" s="27"/>
-      <c r="C15" s="30">
+      <c r="B15" s="24"/>
+      <c r="C15" s="23">
         <f>SUM('🏷️ Catálogo Productos'!K2:K12)</f>
         <v>405000</v>
       </c>
-      <c r="D15" s="27"/>
-      <c r="E15" s="30">
+      <c r="D15" s="24"/>
+      <c r="E15" s="23">
         <f>SUM('🛒 Ventas'!H2:H58)</f>
         <v>0</v>
       </c>
-      <c r="F15" s="27"/>
-      <c r="G15" s="30">
+      <c r="F15" s="24"/>
+      <c r="G15" s="23">
         <f>SUM('🏢 Activos Fijos'!H2:H11)</f>
-        <v>4150000</v>
-      </c>
-      <c r="H15" s="27"/>
+        <v>5650000</v>
+      </c>
+      <c r="H15" s="24"/>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A16" s="27"/>
-      <c r="B16" s="27"/>
-      <c r="C16" s="27"/>
-      <c r="D16" s="27"/>
-      <c r="E16" s="27"/>
-      <c r="F16" s="27"/>
-      <c r="G16" s="27"/>
-      <c r="H16" s="27"/>
+      <c r="A16" s="24"/>
+      <c r="B16" s="24"/>
+      <c r="C16" s="24"/>
+      <c r="D16" s="24"/>
+      <c r="E16" s="24"/>
+      <c r="F16" s="24"/>
+      <c r="G16" s="24"/>
+      <c r="H16" s="24"/>
     </row>
     <row r="19" spans="1:7" ht="17" x14ac:dyDescent="0.4">
       <c r="A19" s="4" t="s">
@@ -1928,14 +1919,6 @@
     </row>
   </sheetData>
   <mergeCells count="24">
-    <mergeCell ref="G15:H16"/>
-    <mergeCell ref="C14:D14"/>
-    <mergeCell ref="E14:F14"/>
-    <mergeCell ref="C9:D9"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="C6:D6"/>
-    <mergeCell ref="E15:F16"/>
-    <mergeCell ref="C5:D5"/>
     <mergeCell ref="A3:D3"/>
     <mergeCell ref="A10:B10"/>
     <mergeCell ref="A1:I1"/>
@@ -1952,6 +1935,14 @@
     <mergeCell ref="C4:D4"/>
     <mergeCell ref="C10:D10"/>
     <mergeCell ref="A7:B7"/>
+    <mergeCell ref="G15:H16"/>
+    <mergeCell ref="C14:D14"/>
+    <mergeCell ref="E14:F14"/>
+    <mergeCell ref="C9:D9"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="C6:D6"/>
+    <mergeCell ref="E15:F16"/>
+    <mergeCell ref="C5:D5"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing r:id="rId1"/>
@@ -5017,7 +5008,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <dimension ref="A1:J35"/>
+  <dimension ref="A1:J26"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="17" customWidth="1"/>
@@ -5069,7 +5060,7 @@
         <v>141</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="C2" s="6" t="s">
         <v>42</v>
@@ -5102,7 +5093,7 @@
         <v>145</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="C3" s="17" t="s">
         <v>42</v>
@@ -5135,7 +5126,7 @@
         <v>147</v>
       </c>
       <c r="B4" s="17" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="C4" s="17" t="s">
         <v>42</v>
@@ -5168,7 +5159,7 @@
         <v>152</v>
       </c>
       <c r="B5" s="17" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="C5" s="17" t="s">
         <v>42</v>
@@ -5193,7 +5184,7 @@
         <v>143</v>
       </c>
       <c r="J5" s="17" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
     </row>
     <row r="6" spans="1:10" ht="20" customHeight="1" x14ac:dyDescent="0.35">
@@ -5209,7 +5200,9 @@
       <c r="D6" s="6" t="s">
         <v>149</v>
       </c>
-      <c r="E6" s="7"/>
+      <c r="E6" s="19">
+        <v>1</v>
+      </c>
       <c r="F6" s="15" t="s">
         <v>41</v>
       </c>
@@ -5218,7 +5211,7 @@
       </c>
       <c r="H6" s="8">
         <f t="shared" ref="H6:H11" si="3">E6*G6</f>
-        <v>0</v>
+        <v>15000</v>
       </c>
       <c r="I6" s="15" t="s">
         <v>150</v>
@@ -5240,7 +5233,9 @@
       <c r="D7" s="17" t="s">
         <v>154</v>
       </c>
-      <c r="E7" s="19"/>
+      <c r="E7" s="19">
+        <v>1</v>
+      </c>
       <c r="F7" s="15" t="s">
         <v>41</v>
       </c>
@@ -5249,7 +5244,7 @@
       </c>
       <c r="H7" s="18">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>45000</v>
       </c>
       <c r="I7" s="16" t="s">
         <v>155</v>
@@ -5271,7 +5266,9 @@
       <c r="D8" s="6" t="s">
         <v>142</v>
       </c>
-      <c r="E8" s="7"/>
+      <c r="E8" s="19">
+        <v>1</v>
+      </c>
       <c r="F8" s="15" t="s">
         <v>41</v>
       </c>
@@ -5280,7 +5277,7 @@
       </c>
       <c r="H8" s="8">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>60000</v>
       </c>
       <c r="I8" s="15" t="s">
         <v>159</v>
@@ -5302,7 +5299,9 @@
       <c r="D9" s="17" t="s">
         <v>129</v>
       </c>
-      <c r="E9" s="19"/>
+      <c r="E9" s="19">
+        <v>1</v>
+      </c>
       <c r="F9" s="15" t="s">
         <v>41</v>
       </c>
@@ -5311,7 +5310,7 @@
       </c>
       <c r="H9" s="18">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>450000</v>
       </c>
       <c r="I9" s="16" t="s">
         <v>163</v>
@@ -5322,7 +5321,7 @@
     </row>
     <row r="10" spans="1:10" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="16" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="B10" s="6" t="s">
         <v>166</v>
@@ -5333,7 +5332,9 @@
       <c r="D10" s="6" t="s">
         <v>167</v>
       </c>
-      <c r="E10" s="7"/>
+      <c r="E10" s="19">
+        <v>1</v>
+      </c>
       <c r="F10" s="15" t="s">
         <v>41</v>
       </c>
@@ -5342,7 +5343,7 @@
       </c>
       <c r="H10" s="8">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>80000</v>
       </c>
       <c r="I10" s="15" t="s">
         <v>168</v>
@@ -5356,7 +5357,7 @@
         <v>174</v>
       </c>
       <c r="B11" s="17" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="C11" s="17" t="s">
         <v>53</v>
@@ -5364,7 +5365,9 @@
       <c r="D11" s="17" t="s">
         <v>142</v>
       </c>
-      <c r="E11" s="19"/>
+      <c r="E11" s="19">
+        <v>1</v>
+      </c>
       <c r="F11" s="15" t="s">
         <v>41</v>
       </c>
@@ -5373,7 +5376,7 @@
       </c>
       <c r="H11" s="18">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>850000</v>
       </c>
       <c r="I11" s="16" t="s">
         <v>171</v>
@@ -5382,148 +5385,184 @@
         <v>172</v>
       </c>
     </row>
-    <row r="12" spans="1:10" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:10" ht="20" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A12" s="15" t="s">
-        <v>175</v>
-      </c>
-      <c r="B12" s="17"/>
-      <c r="C12" s="17"/>
-      <c r="D12" s="17"/>
-      <c r="E12" s="19"/>
-      <c r="F12" s="16"/>
-      <c r="G12" s="18"/>
-      <c r="H12" s="18"/>
-      <c r="I12" s="16"/>
-      <c r="J12" s="23"/>
-    </row>
-    <row r="13" spans="1:10" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+        <v>182</v>
+      </c>
+      <c r="B12" s="9"/>
+      <c r="C12" s="9"/>
+      <c r="D12" s="21" t="s">
+        <v>173</v>
+      </c>
+      <c r="E12" s="10">
+        <f>SUM(E2:E11)</f>
+        <v>13</v>
+      </c>
+      <c r="F12" s="9"/>
+      <c r="G12" s="9"/>
+      <c r="H12" s="11">
+        <f>SUM(H2:H11)</f>
+        <v>5650000</v>
+      </c>
+      <c r="I12" s="9"/>
+      <c r="J12" s="1"/>
+    </row>
+    <row r="13" spans="1:10" ht="20" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A13" s="15" t="s">
-        <v>176</v>
-      </c>
-      <c r="B13" s="17"/>
-      <c r="C13" s="17"/>
-      <c r="D13" s="17"/>
-      <c r="E13" s="19"/>
-      <c r="F13" s="16"/>
-      <c r="G13" s="18"/>
-      <c r="H13" s="18"/>
-      <c r="I13" s="16"/>
-      <c r="J13" s="23"/>
+        <v>183</v>
+      </c>
+      <c r="B13" s="1"/>
+      <c r="C13" s="1"/>
+      <c r="D13" s="1"/>
+      <c r="E13" s="1"/>
+      <c r="F13" s="1"/>
+      <c r="G13" s="1"/>
+      <c r="H13" s="22" t="str">
+        <f t="shared" ref="H13:H26" si="4">IF(E13="","",E13*G13)</f>
+        <v/>
+      </c>
+      <c r="I13" s="1"/>
+      <c r="J13" s="1"/>
     </row>
     <row r="14" spans="1:10" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="15" t="s">
-        <v>177</v>
-      </c>
-      <c r="B14" s="17"/>
-      <c r="C14" s="17"/>
-      <c r="D14" s="17"/>
-      <c r="E14" s="19"/>
-      <c r="F14" s="16"/>
-      <c r="G14" s="18"/>
-      <c r="H14" s="18"/>
-      <c r="I14" s="16"/>
-      <c r="J14" s="23"/>
+        <v>184</v>
+      </c>
+      <c r="B14" s="1"/>
+      <c r="C14" s="1"/>
+      <c r="D14" s="1"/>
+      <c r="E14" s="1"/>
+      <c r="F14" s="1"/>
+      <c r="G14" s="1"/>
+      <c r="H14" s="22" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="I14" s="1"/>
+      <c r="J14" s="1"/>
     </row>
     <row r="15" spans="1:10" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="15" t="s">
-        <v>178</v>
-      </c>
-      <c r="B15" s="17"/>
-      <c r="C15" s="17"/>
-      <c r="D15" s="17"/>
-      <c r="E15" s="19"/>
-      <c r="F15" s="16"/>
-      <c r="G15" s="18"/>
-      <c r="H15" s="18"/>
-      <c r="I15" s="16"/>
-      <c r="J15" s="23"/>
+        <v>185</v>
+      </c>
+      <c r="B15" s="1"/>
+      <c r="C15" s="1"/>
+      <c r="D15" s="1"/>
+      <c r="E15" s="1"/>
+      <c r="F15" s="1"/>
+      <c r="G15" s="1"/>
+      <c r="H15" s="22" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="I15" s="1"/>
+      <c r="J15" s="1"/>
     </row>
     <row r="16" spans="1:10" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="15" t="s">
-        <v>179</v>
-      </c>
-      <c r="B16" s="17"/>
-      <c r="C16" s="17"/>
-      <c r="D16" s="17"/>
-      <c r="E16" s="19"/>
-      <c r="F16" s="16"/>
-      <c r="G16" s="18"/>
-      <c r="H16" s="18"/>
-      <c r="I16" s="16"/>
-      <c r="J16" s="23"/>
+        <v>175</v>
+      </c>
+      <c r="B16" s="1"/>
+      <c r="C16" s="1"/>
+      <c r="D16" s="1"/>
+      <c r="E16" s="1"/>
+      <c r="F16" s="1"/>
+      <c r="G16" s="1"/>
+      <c r="H16" s="22" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="I16" s="1"/>
+      <c r="J16" s="1"/>
     </row>
     <row r="17" spans="1:10" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="15" t="s">
-        <v>180</v>
-      </c>
-      <c r="B17" s="17"/>
-      <c r="C17" s="17"/>
-      <c r="D17" s="17"/>
-      <c r="E17" s="19"/>
-      <c r="F17" s="16"/>
-      <c r="G17" s="18"/>
-      <c r="H17" s="18"/>
-      <c r="I17" s="16"/>
-      <c r="J17" s="23"/>
+        <v>176</v>
+      </c>
+      <c r="B17" s="1"/>
+      <c r="C17" s="1"/>
+      <c r="D17" s="1"/>
+      <c r="E17" s="1"/>
+      <c r="F17" s="1"/>
+      <c r="G17" s="1"/>
+      <c r="H17" s="22" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="I17" s="1"/>
+      <c r="J17" s="1"/>
     </row>
     <row r="18" spans="1:10" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="15" t="s">
-        <v>181</v>
-      </c>
-      <c r="B18" s="17"/>
-      <c r="C18" s="17"/>
-      <c r="D18" s="17"/>
-      <c r="E18" s="19"/>
-      <c r="F18" s="16"/>
-      <c r="G18" s="18"/>
-      <c r="H18" s="18"/>
-      <c r="I18" s="16"/>
-      <c r="J18" s="23"/>
+        <v>177</v>
+      </c>
+      <c r="B18" s="1"/>
+      <c r="C18" s="1"/>
+      <c r="D18" s="1"/>
+      <c r="E18" s="1"/>
+      <c r="F18" s="1"/>
+      <c r="G18" s="1"/>
+      <c r="H18" s="22" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="I18" s="1"/>
+      <c r="J18" s="1"/>
     </row>
     <row r="19" spans="1:10" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" s="15" t="s">
-        <v>182</v>
-      </c>
-      <c r="B19" s="17"/>
-      <c r="C19" s="17"/>
-      <c r="D19" s="19"/>
-      <c r="E19" s="16"/>
-      <c r="F19" s="18"/>
-      <c r="G19" s="18"/>
-      <c r="H19" s="16"/>
-      <c r="I19" s="17"/>
-    </row>
-    <row r="20" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+        <v>178</v>
+      </c>
+      <c r="B19" s="1"/>
+      <c r="C19" s="1"/>
+      <c r="D19" s="1"/>
+      <c r="E19" s="1"/>
+      <c r="F19" s="1"/>
+      <c r="G19" s="1"/>
+      <c r="H19" s="22" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="I19" s="1"/>
+      <c r="J19" s="1"/>
+    </row>
+    <row r="20" spans="1:10" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20" s="15" t="s">
-        <v>183</v>
-      </c>
-      <c r="J20" s="9"/>
-    </row>
-    <row r="21" spans="1:10" ht="20" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+        <v>179</v>
+      </c>
+      <c r="B20" s="1"/>
+      <c r="C20" s="1"/>
+      <c r="D20" s="1"/>
+      <c r="E20" s="1"/>
+      <c r="F20" s="1"/>
+      <c r="G20" s="1"/>
+      <c r="H20" s="22" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="I20" s="1"/>
+      <c r="J20" s="1"/>
+    </row>
+    <row r="21" spans="1:10" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A21" s="15" t="s">
-        <v>184</v>
-      </c>
-      <c r="B21" s="9"/>
-      <c r="C21" s="9"/>
-      <c r="D21" s="21" t="s">
-        <v>173</v>
-      </c>
-      <c r="E21" s="10">
-        <f>SUM(E2:E11)</f>
-        <v>7</v>
-      </c>
-      <c r="F21" s="9"/>
-      <c r="G21" s="9"/>
-      <c r="H21" s="11">
-        <f>SUM(H2:H11)</f>
-        <v>4150000</v>
-      </c>
-      <c r="I21" s="9"/>
+        <v>180</v>
+      </c>
+      <c r="B21" s="1"/>
+      <c r="C21" s="1"/>
+      <c r="D21" s="1"/>
+      <c r="E21" s="1"/>
+      <c r="F21" s="1"/>
+      <c r="G21" s="1"/>
+      <c r="H21" s="22" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="I21" s="1"/>
       <c r="J21" s="1"/>
     </row>
-    <row r="22" spans="1:10" ht="20" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:10" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A22" s="15" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="B22" s="1"/>
       <c r="C22" s="1"/>
@@ -5532,7 +5571,7 @@
       <c r="F22" s="1"/>
       <c r="G22" s="1"/>
       <c r="H22" s="22" t="str">
-        <f t="shared" ref="H22:H35" si="4">IF(E22="","",E22*G22)</f>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="I22" s="1"/>
@@ -5540,7 +5579,7 @@
     </row>
     <row r="23" spans="1:10" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A23" s="15" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="B23" s="1"/>
       <c r="C23" s="1"/>
@@ -5557,7 +5596,7 @@
     </row>
     <row r="24" spans="1:10" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A24" s="15" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="B24" s="1"/>
       <c r="C24" s="1"/>
@@ -5574,7 +5613,7 @@
     </row>
     <row r="25" spans="1:10" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A25" s="15" t="s">
-        <v>177</v>
+        <v>184</v>
       </c>
       <c r="B25" s="1"/>
       <c r="C25" s="1"/>
@@ -5589,9 +5628,9 @@
       <c r="I25" s="1"/>
       <c r="J25" s="1"/>
     </row>
-    <row r="26" spans="1:10" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A26" s="15" t="s">
-        <v>178</v>
+        <v>185</v>
       </c>
       <c r="B26" s="1"/>
       <c r="C26" s="1"/>
@@ -5604,159 +5643,6 @@
         <v/>
       </c>
       <c r="I26" s="1"/>
-      <c r="J26" s="1"/>
-    </row>
-    <row r="27" spans="1:10" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A27" s="15" t="s">
-        <v>179</v>
-      </c>
-      <c r="B27" s="1"/>
-      <c r="C27" s="1"/>
-      <c r="D27" s="1"/>
-      <c r="E27" s="1"/>
-      <c r="F27" s="1"/>
-      <c r="G27" s="1"/>
-      <c r="H27" s="22" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="I27" s="1"/>
-      <c r="J27" s="1"/>
-    </row>
-    <row r="28" spans="1:10" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A28" s="15" t="s">
-        <v>180</v>
-      </c>
-      <c r="B28" s="1"/>
-      <c r="C28" s="1"/>
-      <c r="D28" s="1"/>
-      <c r="E28" s="1"/>
-      <c r="F28" s="1"/>
-      <c r="G28" s="1"/>
-      <c r="H28" s="22" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="I28" s="1"/>
-      <c r="J28" s="1"/>
-    </row>
-    <row r="29" spans="1:10" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A29" s="15" t="s">
-        <v>181</v>
-      </c>
-      <c r="B29" s="1"/>
-      <c r="C29" s="1"/>
-      <c r="D29" s="1"/>
-      <c r="E29" s="1"/>
-      <c r="F29" s="1"/>
-      <c r="G29" s="1"/>
-      <c r="H29" s="22" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="I29" s="1"/>
-      <c r="J29" s="1"/>
-    </row>
-    <row r="30" spans="1:10" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A30" s="15" t="s">
-        <v>182</v>
-      </c>
-      <c r="B30" s="1"/>
-      <c r="C30" s="1"/>
-      <c r="D30" s="1"/>
-      <c r="E30" s="1"/>
-      <c r="F30" s="1"/>
-      <c r="G30" s="1"/>
-      <c r="H30" s="22" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="I30" s="1"/>
-      <c r="J30" s="1"/>
-    </row>
-    <row r="31" spans="1:10" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A31" s="15" t="s">
-        <v>183</v>
-      </c>
-      <c r="B31" s="1"/>
-      <c r="C31" s="1"/>
-      <c r="D31" s="1"/>
-      <c r="E31" s="1"/>
-      <c r="F31" s="1"/>
-      <c r="G31" s="1"/>
-      <c r="H31" s="22" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="I31" s="1"/>
-      <c r="J31" s="1"/>
-    </row>
-    <row r="32" spans="1:10" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A32" s="15" t="s">
-        <v>184</v>
-      </c>
-      <c r="B32" s="1"/>
-      <c r="C32" s="1"/>
-      <c r="D32" s="1"/>
-      <c r="E32" s="1"/>
-      <c r="F32" s="1"/>
-      <c r="G32" s="1"/>
-      <c r="H32" s="22" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="I32" s="1"/>
-      <c r="J32" s="1"/>
-    </row>
-    <row r="33" spans="1:10" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A33" s="15" t="s">
-        <v>185</v>
-      </c>
-      <c r="B33" s="1"/>
-      <c r="C33" s="1"/>
-      <c r="D33" s="1"/>
-      <c r="E33" s="1"/>
-      <c r="F33" s="1"/>
-      <c r="G33" s="1"/>
-      <c r="H33" s="22" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="I33" s="1"/>
-      <c r="J33" s="1"/>
-    </row>
-    <row r="34" spans="1:10" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A34" s="15" t="s">
-        <v>186</v>
-      </c>
-      <c r="B34" s="1"/>
-      <c r="C34" s="1"/>
-      <c r="D34" s="1"/>
-      <c r="E34" s="1"/>
-      <c r="F34" s="1"/>
-      <c r="G34" s="1"/>
-      <c r="H34" s="22" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="I34" s="1"/>
-      <c r="J34" s="1"/>
-    </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A35" s="15" t="s">
-        <v>187</v>
-      </c>
-      <c r="B35" s="1"/>
-      <c r="C35" s="1"/>
-      <c r="D35" s="1"/>
-      <c r="E35" s="1"/>
-      <c r="F35" s="1"/>
-      <c r="G35" s="1"/>
-      <c r="H35" s="22" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="I35" s="1"/>
     </row>
   </sheetData>
   <phoneticPr fontId="11" type="noConversion"/>
@@ -5768,13 +5654,13 @@
           <x14:formula1>
             <xm:f>'⚙️ Configuración'!$I$4:$I$8</xm:f>
           </x14:formula1>
-          <xm:sqref>C21:C39 B19 C2:C18</xm:sqref>
+          <xm:sqref>C12:C30 C2:C11</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" xr:uid="{00000000-0002-0000-0500-000001000000}">
           <x14:formula1>
             <xm:f>'⚙️ Configuración'!$G$4:$G$7</xm:f>
           </x14:formula1>
-          <xm:sqref>F21:F39 E19 F2:F18</xm:sqref>
+          <xm:sqref>F12:F30 F2:F11</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>

</xml_diff>